<commit_message>
CardTable.xlsx를 한글 cards.json과 일치하도록 재생성
CardTable.xlsx가 영문 샘플로 남아 있어, 익스포터를 돌리면 커밋된 한글
cards.json이 영문으로 되돌아가는 불일치가 있었다. cards.json을 원본으로
삼아 워크북을 다시 만들어, 라운드트립 익스포트 시 cards.json이 그대로
재현되도록 맞췄다.

주요 변경
- CardTable.xlsx를 한글 데이터(베기/방어/집중/강타)로 재생성.
- create_card_table.py 추가: cards.json을 읽어 CardTable.xlsx를 생성하는
  스크립트. 이후 카드 문구 수정은 xlsx를 원본으로 편집한다.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/project-a/tables/excel/CardTable.xlsx
+++ b/project-a/tables/excel/CardTable.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="cards" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="cards" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -418,10 +418,10 @@
   <cols>
     <col width="18" customWidth="1" min="2" max="2"/>
     <col width="18" customWidth="1" min="3" max="3"/>
-    <col width="10" customWidth="1" min="4" max="4"/>
-    <col width="34" customWidth="1" min="5" max="5"/>
-    <col width="14" customWidth="1" min="6" max="6"/>
-    <col width="18" customWidth="1" min="7" max="7"/>
+    <col width="8" customWidth="1" min="4" max="4"/>
+    <col width="40" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="16" customWidth="1" min="7" max="7"/>
     <col width="62" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
@@ -550,7 +550,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Slash</t>
+          <t>베기</t>
         </is>
       </c>
       <c r="D5" t="n">
@@ -558,7 +558,7 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Deal 6 damage.</t>
+          <t>피해 6을 줍니다.</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
@@ -583,7 +583,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Guard</t>
+          <t>방어</t>
         </is>
       </c>
       <c r="D6" t="n">
@@ -591,7 +591,7 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Gain 7 block.</t>
+          <t>방어도 7을 얻습니다.</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
@@ -616,7 +616,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Focus</t>
+          <t>집중</t>
         </is>
       </c>
       <c r="D7" t="n">
@@ -624,7 +624,7 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Draw 1 card. Gain 1 energy.</t>
+          <t>카드 1장을 뽑고 에너지 1을 얻습니다.</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
@@ -649,7 +649,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Heavy Slash</t>
+          <t>강타</t>
         </is>
       </c>
       <c r="D8" t="n">
@@ -657,7 +657,7 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Deal 12 damage.</t>
+          <t>피해 12를 줍니다.</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">

</xml_diff>